<commit_message>
Updated file with September seminar
</commit_message>
<xml_diff>
--- a/data/upcoming.xlsx
+++ b/data/upcoming.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sigrid\Documents\BES\work\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sigrid\Documents\BES\BES_new\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="8145"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11715"/>
   </bookViews>
   <sheets>
     <sheet name="Conferences" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>date</t>
   </si>
@@ -49,22 +49,10 @@
     <t>Seminar</t>
   </si>
   <si>
-    <t>https://urldefense.com/v3/__https:/forms.gle/GDwwEaYVp94ohZ6E8__;!!I5RyydYb1W3tjTUU!xg6uNk_Ygi0ta18SLPbwtKdkU58aQ7yQN9nwtPpUMDYMivd3pVICCdVnc6JYK4HxLxshFmAX4declb3TqP_F6GeZo1rt$</t>
+    <t xml:space="preserve"> https://forms.gle/SEmmrAe1qzwLsh1y8</t>
   </si>
   <si>
-    <t>Real-World Data Quality - Assessing data quality and demonstrating fitness-for-purpose</t>
-  </si>
-  <si>
-    <t>RWD Frameworks: Estimands,  Target Trial Framework</t>
-  </si>
-  <si>
-    <t>https://forms.gle/mKf5iYAfTVNbMzrL7</t>
-  </si>
-  <si>
-    <t>Methods for rare diseases, small or special populations</t>
-  </si>
-  <si>
-    <t>https://forms.gle/y96E9KkUNqYgKbJv7</t>
+    <t>Zooming in on feasibility assessments and data quality</t>
   </si>
 </sst>
 </file>
@@ -125,7 +113,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -160,7 +148,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -185,7 +172,7 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="9525" cy="9525"/>
@@ -194,7 +181,7 @@
         <xdr:cNvPr id="2" name="image1.gif" descr="https://ssl.gstatic.com/ui/v1/icons/mail/images/cleardot.gif">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -219,7 +206,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="9525" cy="9525"/>
@@ -228,7 +215,7 @@
         <xdr:cNvPr id="3" name="image1.gif" descr="https://ssl.gstatic.com/ui/v1/icons/mail/images/cleardot.gif">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -519,7 +506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D943"/>
+  <dimension ref="A1:D941"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" style="8" bestFit="1" customWidth="1"/>
@@ -545,8 +532,8 @@
     </row>
     <row r="2" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="str">
-        <f>"15.03.2023"</f>
-        <v>15.03.2023</v>
+        <f>"16.09.2026"</f>
+        <v>16.09.2026</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>6</v>
@@ -558,35 +545,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="str">
-        <f>"27.10.2023"</f>
-        <v>27.10.2023</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="str">
-        <f>"13.06.2024"</f>
-        <v>13.06.2024</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>10</v>
-      </c>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="7"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="7"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
@@ -619,12 +586,12 @@
       <c r="C10" s="1"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
+      <c r="A11" s="2"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
+      <c r="A12" s="2"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
@@ -689,19 +656,19 @@
       <c r="C24" s="1"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="2"/>
+      <c r="A25" s="9"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="2"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
+      <c r="A26" s="9"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="9"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="9"/>
@@ -745,13 +712,13 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="9"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="9"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="9"/>
@@ -765,8 +732,8 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="9"/>
-      <c r="B40" s="9"/>
-      <c r="C40" s="9"/>
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="9"/>
@@ -775,8 +742,8 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
+      <c r="B42" s="9"/>
+      <c r="C42" s="9"/>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="9"/>
@@ -810,13 +777,13 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="9"/>
-      <c r="B49" s="9"/>
-      <c r="C49" s="9"/>
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="9"/>
-      <c r="B50" s="9"/>
-      <c r="C50" s="9"/>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="9"/>
@@ -1379,14 +1346,14 @@
       <c r="C162" s="4"/>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A163" s="9"/>
-      <c r="B163" s="4"/>
-      <c r="C163" s="4"/>
+      <c r="A163" s="10"/>
+      <c r="B163" s="5"/>
+      <c r="C163" s="5"/>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A164" s="9"/>
-      <c r="B164" s="4"/>
-      <c r="C164" s="4"/>
+      <c r="A164" s="10"/>
+      <c r="B164" s="5"/>
+      <c r="C164" s="5"/>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" s="10"/>
@@ -5273,23 +5240,12 @@
       <c r="B941" s="5"/>
       <c r="C941" s="5"/>
     </row>
-    <row r="942" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A942" s="10"/>
-      <c r="B942" s="5"/>
-      <c r="C942" s="5"/>
-    </row>
-    <row r="943" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A943" s="10"/>
-      <c r="B943" s="5"/>
-      <c r="C943" s="5"/>
-    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D3" r:id="rId1"/>
-    <hyperlink ref="D4" r:id="rId2"/>
+    <hyperlink ref="D2" r:id="rId1" display="https://forms.gle/y96E9KkUNqYgKbJv7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
-  <drawing r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>